<commit_message>
feat(radar): atualizar sinais e liquidacoes 06/10 com jogo noturno Ponte Preta x Juventude
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-06.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-06.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -509,26 +509,6 @@
           <t>Liquidez_Lay</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Hora_Str</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Risco_Red_R$</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Stake_Sugerida_R$</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Lucro_Green_R$</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -601,20 +581,6 @@
       <c r="P2" t="n">
         <v>161</v>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="R2" t="n">
-        <v>200</v>
-      </c>
-      <c r="S2" t="n">
-        <v>11.11</v>
-      </c>
-      <c r="T2" t="n">
-        <v>10.61</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -687,20 +653,6 @@
       <c r="P3" t="n">
         <v>271</v>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
-        <v>200</v>
-      </c>
-      <c r="S3" t="n">
-        <v>11.43</v>
-      </c>
-      <c r="T3" t="n">
-        <v>10.92</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -773,19 +725,73 @@
       <c r="P4" t="n">
         <v>257</v>
       </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>200</v>
-      </c>
-      <c r="S4" t="n">
-        <v>33.33</v>
-      </c>
-      <c r="T4" t="n">
-        <v>31.83</v>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Brazilian Serie B</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ponte Preta x Juventude</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ponte Preta</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Juventude</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>coletor (KO-10)</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>707</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(forward): atualiza resultados e liquidacoes ate 10/10/2026 e sincroniza forward ledger
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-06.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-10-06.xlsx
@@ -630,15 +630,19 @@
       <c r="K3" t="n">
         <v>1.29</v>
       </c>
-      <c r="L3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
+          <t>✅ LIQUIDADO</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">

</xml_diff>